<commit_message>
Add allergy and intolerance codes to valueset 88dafdbd895cd510dac51a54ac8bc5bb538ec70e
</commit_message>
<xml_diff>
--- a/nr-doc-core-allergy-intolerance/ig/ValueSet-fr-core-vs-allergy-intolerance-type.xlsx
+++ b/nr-doc-core-allergy-intolerance/ig/ValueSet-fr-core-vs-allergy-intolerance-type.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Include #0" r:id="rId4" sheetId="2"/>
+    <sheet name="Include #1" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="41">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-31T13:13:23+00:00</t>
+    <t>2026-07-31T13:21:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -105,6 +106,24 @@
     <t>Concept</t>
   </si>
   <si>
+    <t>allergy</t>
+  </si>
+  <si>
+    <t>allergie</t>
+  </si>
+  <si>
+    <t>intolerance</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>System URI</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/allergy-intolerance-type</t>
+  </si>
+  <si>
     <t>56840009</t>
   </si>
   <si>
@@ -115,12 +134,6 @@
   </si>
   <si>
     <t>hypersensibilité non allergique</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>System URI</t>
   </si>
   <si>
     <t>http://snomed.info/sct</t>
@@ -423,23 +436,77 @@
         <v>32</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s" s="2">
         <v>35</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="30.703125" customWidth="true"/>
+    <col min="2" max="2" width="50.703125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>34</v>
+      </c>
       <c r="B5" t="s" s="2">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>